<commit_message>
Feat: Carga masiva de estados reproductivos
Pruebo descripciones de copilot:
Add endpoint POST /api/v1/animales/estado-reproductivo/csv and support for bulk importing reproductive states. Introduces CargaMasivaEstadoResponse DTO and updates EstadoReproductivoCsvRequest to use animalId (Long). Implements cargarEstadosMasivo in AnimalServiceImpl (transactional) using EstadoReproductivoCsvService to parse/validate, persist EstadoReproductivo entries, enforce productor/establecimiento membership and active-animal checks, and return processed/exitosos/fallidos with error rows. Update EstadoReproductivoCsvServiceImpl parsing/validation (expect numeric IdAnimal and updated error messages), small ExcelReader validation tweak, repository addition (findByIdCaravanaOficial), tests and import templates updated accordingly.
</commit_message>
<xml_diff>
--- a/docs/TemplateCargaEstados.xlsx
+++ b/docs/TemplateCargaEstados.xlsx
@@ -6,54 +6,36 @@
     <workbookView activeTab="0"/>
   </bookViews>
   <sheets>
-    <sheet name="Estados" r:id="rId3" sheetId="1"/>
+    <sheet name="Animales" r:id="rId3" sheetId="1"/>
   </sheets>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
   <si>
-    <t>IdCaravana</t>
+    <t>IdAnimal</t>
   </si>
   <si>
-    <t>Estado (VACIA/GESTANTE/CELO/ANESTRO)</t>
+    <t>Estado</t>
   </si>
   <si>
-    <t>FechaUltimoParto (AAAA-MM-DD)</t>
+    <t>FechaUltimoParto</t>
   </si>
   <si>
-    <t>FechaUltimaInseminacion (AAAA-MM-DD)</t>
+    <t>FechaUltimaInseminacion</t>
   </si>
   <si>
-    <t>X-123</t>
+    <t>123</t>
   </si>
   <si>
     <t>GESTANTE</t>
   </si>
   <si>
-    <t>2023-05-10</t>
+    <t>2023-01-01</t>
   </si>
   <si>
-    <t>2023-08-15</t>
-  </si>
-  <si>
-    <t>X-124</t>
-  </si>
-  <si>
-    <t>VACIA</t>
-  </si>
-  <si>
-    <t/>
-  </si>
-  <si>
-    <t>X-125</t>
-  </si>
-  <si>
-    <t>CELO</t>
-  </si>
-  <si>
-    <t>2023-11-20</t>
+    <t>2023-02-01</t>
   </si>
 </sst>
 </file>
@@ -98,7 +80,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:D4"/>
+  <dimension ref="A1:D2"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -129,34 +111,6 @@
         <v>7</v>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" t="s" s="0">
-        <v>8</v>
-      </c>
-      <c r="B3" t="s" s="0">
-        <v>9</v>
-      </c>
-      <c r="C3" t="s" s="0">
-        <v>10</v>
-      </c>
-      <c r="D3" t="s" s="0">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="s" s="0">
-        <v>11</v>
-      </c>
-      <c r="B4" t="s" s="0">
-        <v>12</v>
-      </c>
-      <c r="C4" t="s" s="0">
-        <v>10</v>
-      </c>
-      <c r="D4" t="s" s="0">
-        <v>13</v>
-      </c>
-    </row>
   </sheetData>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>

</xml_diff>